<commit_message>
Bug status sheet: results from the dev server run.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/PTW_Bug_Status_2026-09-29.xlsx
+++ b/docs/qa/PTW_Bug_Status_2026-09-29.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">PTW bug lists – consolidated status</t>
   </si>
   <si>
-    <t xml:space="preserve">Build: branch dev_ram (after 2c2473f) with the fixes in this round. Checked 29 Sep 2026.</t>
+    <t xml:space="preserve">Build: dev_ram 59e0ccb, deployed to http://200.234.45.51 on 29 Sep 2026; automated checks run against the dev server.</t>
   </si>
   <si>
     <t xml:space="preserve">Items in both lists</t>
@@ -96,13 +96,13 @@
     <t xml:space="preserve">Passed automated UI test</t>
   </si>
   <si>
-    <t xml:space="preserve">Playwright run against local build (17 checks, all passed)</t>
+    <t xml:space="preserve">Playwright against the dev server (19 checks incl. plain-HTTP copy and notification link, all passed)</t>
   </si>
   <si>
     <t xml:space="preserve">Passed automated API test</t>
   </si>
   <si>
-    <t xml:space="preserve">API run against local build (7 checks, all passed)</t>
+    <t xml:space="preserve">API checks against the dev server (7 checks, all passed)</t>
   </si>
   <si>
     <t xml:space="preserve">Passed unit test</t>
@@ -138,7 +138,7 @@
     <t xml:space="preserve">Items marked “retest on dev server” must be checked on http://200.234.45.51 after the next deployment, not on localhost: several causes only appear on plain HTTP.</t>
   </si>
   <si>
-    <t xml:space="preserve">Some fixes need the database migrations 0047 (certificate start date) and 0048 (role-change message) on the server; see “Deployment notes”.</t>
+    <t xml:space="preserve">Migrations 0047 and 0048 are applied on the dev server.</t>
   </si>
   <si>
     <t xml:space="preserve">Example: row OI-15 → retest by adding an employee with +91 and a 10-digit number → put “Pass” in M.</t>
@@ -243,7 +243,7 @@
     <t xml:space="preserve">Root cause: the dev server is plain HTTP, where browsers disable crypto.randomUUID; new section/field ids used it. Replaced with an id generator that works on HTTP.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass – automated UI test (local); Fixed – retest on dev server</t>
+    <t xml:space="preserve">Pass – automated UI test (dev server)</t>
   </si>
   <si>
     <t xml:space="preserve">Must be retested on the dev server (HTTP) – localhost is treated as secure.</t>
@@ -285,9 +285,6 @@
     <t xml:space="preserve">Root cause: after reporting, the app opened /incidents/undefined and the server replied 'Validation failed (uuid is expected)', read as 'UUID expired'. Report now opens the new record.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass – automated UI test (local)</t>
-  </si>
-  <si>
     <t xml:space="preserve">D3-06</t>
   </si>
   <si>
@@ -321,222 +318,225 @@
     <t xml:space="preserve">Root cause: messages with the same wording about different permits were merged, and a merged entry linked to the permit list. Messages now merge only when they are about the same record, so each opens its own permit.</t>
   </si>
   <si>
+    <t xml:space="preserve">D3-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Creation – LOTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add Lockout/Tagout is not working while creating a permit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Add LOTOTO' stays unavailable until the chosen machine has a LOTOTO plan. The hint now links to create a plan for that machine (opens in a new tab) and a 'refresh the list' action; LOTOTO rows can be removed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retest with a machine that has an approved LOTOTO plan and one that has none.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Closure – Evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After adding evidence during permit closure, "Authentication required" is displayed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root cause: file uploads skipped the sign-in refresh, so after the 5-minute session token expired they failed with 'Authentication required'. All uploads now refresh the session like other requests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retest: stay on the closure page for more than 5 minutes, then add evidence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profile picture cannot be removed, and the selected profile picture does not display.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-47, OI-48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added 'Remove picture' (server and settings page). Picture display fixed by the storage-link fix (D3-02).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass – automated API test (dev server)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uploaded evidence cannot be opened/viewed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-08, OI-67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storage-link fix (D3-02). Incident evidence now lists files that open on click (new download link endpoint).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOD Notification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOD does not receive a notification when the Job Issuer submits a permit and HOD approval is the next step.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-32, OI-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nothing notified approvers on submit. Now, on submit, resubmit and each approval stage, the people holding the next approver role (HOD scoped to their department) get 'Permit waiting for your approval', linking to the permit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User &amp; Roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temporary Password – Copy button is not working.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-39, OI-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root cause: the browser clipboard API is disabled on plain-HTTP sites. Copy now falls back to a method that works on HTTP and shows 'Temporary password copied'. Copy also added where workforce logins are created.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass – automated UI test (dev server, plain HTTP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must be retested on the dev server (HTTP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Download</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Download option is required/available for downloading the details; expected behaviour should be verified.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reports are shown on screen (per product decision). Permits print or save as PDF from 'Print this permit'. Evidence files open/download from the record.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tell us which specific download is still needed, if any.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incident – Root Cause</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clicking Record Root Cause for an unsafe incident does not open the expected popup/form.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Investigation panel rebuilt: root cause form is visible once an investigator is assigned, recorded root causes are listed, each step confirms with a message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incident – Corrective Action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clicking Corrective Action does not open the expected popup/form.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrective action form with owner and due date; added actions are listed with status, 'Mark complete' and 'Cancel action', and a confirmation message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incident – Assign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Manager Incidents, clicking Assign results in "Unable to load page."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The separate manager page is gone; investigators are assigned on the incident page itself. People listed are sign-in accounts so the investigator sees the task.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Creation – Back</t>
+  </si>
+  <si>
+    <t xml:space="preserve">There is no Back button while creating a permit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create/Edit permit now has the standard back link (to Permits, or to the permit when editing).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Page – Back</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Permit page does not have a Back button.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permits is a top-level menu page (no parent to go back to). Every page below it (permit details, edit, journey) has the back link.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Creation – Next</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After entering Basic Information, the Next button does not respond on the first click; user has to click again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root cause: the first Next saved the draft and navigated to the edit page, reloading the wizard on step 1. The address now updates without reloading, so Next moves on first click.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev_vinesh open issues (xlsx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OI-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organization Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description accepts unrestricted special characters and links.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descriptions must be written in words and cannot contain links (server check on organisation records; error shown on the form).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fixed – code review; retest</t>
   </si>
   <si>
-    <t xml:space="preserve">D3-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Creation – LOTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add Lockout/Tagout is not working while creating a permit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Add LOTOTO' stays unavailable until the chosen machine has a LOTOTO plan. The hint now links to create a plan for that machine (opens in a new tab) and a 'refresh the list' action; LOTOTO rows can be removed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retest with a machine that has an approved LOTOTO plan and one that has none.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Closure – Evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">After adding evidence during permit closure, "Authentication required" is displayed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root cause: file uploads skipped the sign-in refresh, so after the 5-minute session token expired they failed with 'Authentication required'. All uploads now refresh the session like other requests.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retest: stay on the closure page for more than 5 minutes, then add evidence.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profile picture cannot be removed, and the selected profile picture does not display.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OI-47, OI-48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Added 'Remove picture' (server and settings page). Picture display fixed by the storage-link fix (D3-02).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pass – automated API test (local)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uploaded evidence cannot be opened/viewed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OI-08, OI-67</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Storage-link fix (D3-02). Incident evidence now lists files that open on click (new download link endpoint).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOD Notification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOD does not receive a notification when the Job Issuer submits a permit and HOD approval is the next step.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OI-32, OI-64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nothing notified approvers on submit. Now, on submit, resubmit and each approval stage, the people holding the next approver role (HOD scoped to their department) get 'Permit waiting for your approval', linking to the permit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User &amp; Roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Temporary Password – Copy button is not working.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OI-39, OI-40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root cause: the browser clipboard API is disabled on plain-HTTP sites. Copy now falls back to a method that works on HTTP and shows 'Temporary password copied'. Copy also added where workforce logins are created.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must be retested on the dev server (HTTP).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Download</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Download option is required/available for downloading the details; expected behaviour should be verified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reports are shown on screen (per product decision). Permits print or save as PDF from 'Print this permit'. Evidence files open/download from the record.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n/a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tell us which specific download is still needed, if any.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incident – Root Cause</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clicking Record Root Cause for an unsafe incident does not open the expected popup/form.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OI-33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Investigation panel rebuilt: root cause form is visible once an investigator is assigned, recorded root causes are listed, each step confirms with a message.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incident – Corrective Action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clicking Corrective Action does not open the expected popup/form.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OI-34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrective action form with owner and due date; added actions are listed with status, 'Mark complete' and 'Cancel action', and a confirmation message.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incident – Assign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Manager Incidents, clicking Assign results in "Unable to load page."</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The separate manager page is gone; investigators are assigned on the incident page itself. People listed are sign-in accounts so the investigator sees the task.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Creation – Back</t>
-  </si>
-  <si>
-    <t xml:space="preserve">There is no Back button while creating a permit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create/Edit permit now has the standard back link (to Permits, or to the permit when editing).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Page – Back</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Permit page does not have a Back button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permits is a top-level menu page (no parent to go back to). Every page below it (permit details, edit, journey) has the back link.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Creation – Next</t>
-  </si>
-  <si>
-    <t xml:space="preserve">After entering Basic Information, the Next button does not respond on the first click; user has to click again.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root cause: the first Next saved the draft and navigated to the edit page, reloading the wizard on step 1. The address now updates without reloading, so Next moves on first click.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dev_vinesh open issues (xlsx)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OI-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Organization Management</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description accepts unrestricted special characters and links.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descriptions must be written in words and cannot contain links (server check on organisation records; error shown on the form).</t>
-  </si>
-  <si>
     <t xml:space="preserve">OI-02</t>
   </si>
   <si>
@@ -567,7 +567,7 @@
     <t xml:space="preserve">Active / Archived toggle on Workflows (also Plants, Departments, Locations) lists archived records with the archive date.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass – automated UI test (local) (Locations; same component)</t>
+    <t xml:space="preserve">Pass – automated UI test (dev server) (Locations; same component)</t>
   </si>
   <si>
     <t xml:space="preserve">OI-04</t>
@@ -714,7 +714,7 @@
     <t xml:space="preserve">Names must contain letters (numbers alone refused) – on the form and on the server.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass – automated UI test (local); Pass – automated API test (local)</t>
+    <t xml:space="preserve">Pass – automated UI test (dev server); Pass – automated API test (dev server)</t>
   </si>
   <si>
     <t xml:space="preserve">OI-15</t>
@@ -837,7 +837,7 @@
     <t xml:space="preserve">Competencies now have Delete (and Edit).</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass – automated UI test (local) (same component as certificates)</t>
+    <t xml:space="preserve">Pass – automated UI test (dev server) (same component as certificates)</t>
   </si>
   <si>
     <t xml:space="preserve">OI-25</t>
@@ -2050,7 +2050,7 @@
       </c>
       <c r="B20" s="3" t="n">
         <f aca="false">COUNTIF('Consolidated Bugs'!K2:K91,"*automated UI*")</f>
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>23</v>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="B23" s="3" t="n">
         <f aca="false">COUNTIF('Consolidated Bugs'!K2:K91,"*retest*")+COUNTIF('Consolidated Bugs'!K2:K91,"Retest*")</f>
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>28</v>
@@ -2424,7 +2424,7 @@
         <v>85</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L6" s="9"/>
       <c r="M6" s="10"/>
@@ -2438,16 +2438,16 @@
         <v>51</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>89</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>90</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>64</v>
@@ -2457,13 +2457,13 @@
         <v>7</v>
       </c>
       <c r="J7" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="K7" s="9" t="s">
+      <c r="L7" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="L7" s="9" t="s">
-        <v>93</v>
       </c>
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
@@ -2476,13 +2476,13 @@
         <v>51</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="E8" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>55</v>
@@ -2495,10 +2495,10 @@
         <v>7</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="L8" s="9"/>
       <c r="M8" s="10"/>
@@ -2512,13 +2512,13 @@
         <v>51</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>55</v>
@@ -2531,13 +2531,13 @@
         <v>7</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="K9" s="9" t="s">
         <v>66</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
@@ -2550,13 +2550,13 @@
         <v>51</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>106</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>55</v>
@@ -2569,13 +2569,13 @@
         <v>7</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="K10" s="9" t="s">
         <v>66</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M10" s="10"/>
       <c r="N10" s="10"/>
@@ -2588,31 +2588,31 @@
         <v>51</v>
       </c>
       <c r="C11" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="G11" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="I11" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J11" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="G11" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="H11" s="9" t="s">
+      <c r="K11" s="9" t="s">
         <v>113</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>115</v>
       </c>
       <c r="L11" s="9"/>
       <c r="M11" s="10"/>
@@ -2626,13 +2626,13 @@
         <v>51</v>
       </c>
       <c r="C12" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E12" s="9" t="s">
         <v>116</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>118</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>55</v>
@@ -2641,16 +2641,16 @@
         <v>64</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I12" s="9" t="s">
         <v>7</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L12" s="9"/>
       <c r="M12" s="10"/>
@@ -2664,13 +2664,13 @@
         <v>51</v>
       </c>
       <c r="C13" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>121</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>123</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>55</v>
@@ -2679,16 +2679,16 @@
         <v>64</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I13" s="9" t="s">
         <v>7</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L13" s="9"/>
       <c r="M13" s="10"/>
@@ -2702,13 +2702,13 @@
         <v>51</v>
       </c>
       <c r="C14" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>126</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>128</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>55</v>
@@ -2717,19 +2717,19 @@
         <v>64</v>
       </c>
       <c r="H14" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="K14" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="I14" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="J14" s="9" t="s">
+      <c r="L14" s="9" t="s">
         <v>130</v>
-      </c>
-      <c r="K14" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="L14" s="9" t="s">
-        <v>131</v>
       </c>
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
@@ -2742,16 +2742,16 @@
         <v>51</v>
       </c>
       <c r="C15" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="E15" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="E15" s="9" t="s">
-        <v>134</v>
-      </c>
       <c r="F15" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>12</v>
@@ -2761,13 +2761,13 @@
         <v>12</v>
       </c>
       <c r="J15" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="K15" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="K15" s="9" t="s">
+      <c r="L15" s="9" t="s">
         <v>136</v>
-      </c>
-      <c r="L15" s="9" t="s">
-        <v>137</v>
       </c>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
@@ -2780,13 +2780,13 @@
         <v>51</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>139</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>140</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>55</v>
@@ -2795,16 +2795,16 @@
         <v>64</v>
       </c>
       <c r="H16" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J16" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="I16" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="J16" s="9" t="s">
-        <v>142</v>
-      </c>
       <c r="K16" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L16" s="9"/>
       <c r="M16" s="10"/>
@@ -2818,13 +2818,13 @@
         <v>51</v>
       </c>
       <c r="C17" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="D17" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="E17" s="9" t="s">
         <v>144</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>145</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>55</v>
@@ -2833,16 +2833,16 @@
         <v>64</v>
       </c>
       <c r="H17" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J17" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="I17" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="J17" s="9" t="s">
-        <v>147</v>
-      </c>
       <c r="K17" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L17" s="9"/>
       <c r="M17" s="10"/>
@@ -2856,13 +2856,13 @@
         <v>51</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="E18" s="9" t="s">
         <v>149</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>150</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>55</v>
@@ -2875,10 +2875,10 @@
         <v>7</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L18" s="9"/>
       <c r="M18" s="10"/>
@@ -2892,16 +2892,16 @@
         <v>51</v>
       </c>
       <c r="C19" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="E19" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="E19" s="9" t="s">
-        <v>154</v>
-      </c>
       <c r="F19" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>64</v>
@@ -2911,10 +2911,10 @@
         <v>7</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L19" s="9"/>
       <c r="M19" s="10"/>
@@ -2928,29 +2928,29 @@
         <v>51</v>
       </c>
       <c r="C20" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="E20" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="F20" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G20" s="9" t="s">
         <v>158</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>159</v>
       </c>
       <c r="H20" s="9"/>
       <c r="I20" s="9" t="s">
         <v>12</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L20" s="9"/>
       <c r="M20" s="10"/>
@@ -2964,13 +2964,13 @@
         <v>51</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="E21" s="9" t="s">
         <v>162</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>163</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>55</v>
@@ -2983,10 +2983,10 @@
         <v>7</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L21" s="9"/>
       <c r="M21" s="10"/>
@@ -2997,16 +2997,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="D22" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="E22" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9" t="s">
@@ -3017,10 +3017,10 @@
         <v>7</v>
       </c>
       <c r="J22" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="K22" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="K22" s="9" t="s">
-        <v>98</v>
       </c>
       <c r="L22" s="9"/>
       <c r="M22" s="10"/>
@@ -3031,7 +3031,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>170</v>
@@ -3060,12 +3060,12 @@
       <c r="M23" s="10"/>
       <c r="N23" s="10"/>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>176</v>
@@ -3099,7 +3099,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>181</v>
@@ -3122,7 +3122,7 @@
         <v>184</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L25" s="9"/>
       <c r="M25" s="10"/>
@@ -3133,7 +3133,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>185</v>
@@ -3158,7 +3158,7 @@
         <v>189</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L26" s="9"/>
       <c r="M26" s="10"/>
@@ -3169,7 +3169,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>190</v>
@@ -3194,7 +3194,7 @@
         <v>194</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L27" s="9"/>
       <c r="M27" s="10"/>
@@ -3205,7 +3205,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>195</v>
@@ -3228,7 +3228,7 @@
         <v>198</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L28" s="9"/>
       <c r="M28" s="10"/>
@@ -3239,7 +3239,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>199</v>
@@ -3255,7 +3255,7 @@
         <v>64</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I29" s="9" t="s">
         <v>202</v>
@@ -3264,7 +3264,7 @@
         <v>203</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L29" s="9"/>
       <c r="M29" s="10"/>
@@ -3275,7 +3275,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>204</v>
@@ -3298,7 +3298,7 @@
         <v>207</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L30" s="9"/>
       <c r="M30" s="10"/>
@@ -3309,7 +3309,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>208</v>
@@ -3332,7 +3332,7 @@
         <v>211</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L31" s="9"/>
       <c r="M31" s="10"/>
@@ -3343,7 +3343,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>212</v>
@@ -3379,13 +3379,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>216</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>217</v>
@@ -3413,7 +3413,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>220</v>
@@ -3436,18 +3436,18 @@
         <v>223</v>
       </c>
       <c r="K34" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L34" s="9"/>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>224</v>
@@ -3483,7 +3483,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C36" s="9" t="s">
         <v>230</v>
@@ -3508,7 +3508,7 @@
         <v>234</v>
       </c>
       <c r="K36" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L36" s="9"/>
       <c r="M36" s="10"/>
@@ -3519,7 +3519,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C37" s="9" t="s">
         <v>235</v>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H37" s="9"/>
       <c r="I37" s="9" t="s">
@@ -3542,7 +3542,7 @@
         <v>238</v>
       </c>
       <c r="K37" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L37" s="9"/>
       <c r="M37" s="10"/>
@@ -3553,7 +3553,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>239</v>
@@ -3578,7 +3578,7 @@
         <v>242</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L38" s="9"/>
       <c r="M38" s="10"/>
@@ -3589,7 +3589,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>243</v>
@@ -3612,7 +3612,7 @@
         <v>246</v>
       </c>
       <c r="K39" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L39" s="9"/>
       <c r="M39" s="10"/>
@@ -3623,7 +3623,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>247</v>
@@ -3646,7 +3646,7 @@
         <v>249</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L40" s="9"/>
       <c r="M40" s="10"/>
@@ -3657,7 +3657,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>250</v>
@@ -3680,7 +3680,7 @@
         <v>253</v>
       </c>
       <c r="K41" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L41" s="9"/>
       <c r="M41" s="10"/>
@@ -3691,7 +3691,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C42" s="9" t="s">
         <v>254</v>
@@ -3714,7 +3714,7 @@
         <v>257</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L42" s="9"/>
       <c r="M42" s="10"/>
@@ -3725,7 +3725,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>258</v>
@@ -3750,7 +3750,7 @@
         <v>261</v>
       </c>
       <c r="K43" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L43" s="9"/>
       <c r="M43" s="10"/>
@@ -3761,7 +3761,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C44" s="9" t="s">
         <v>262</v>
@@ -3784,18 +3784,18 @@
         <v>265</v>
       </c>
       <c r="K44" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L44" s="9"/>
       <c r="M44" s="10"/>
       <c r="N44" s="10"/>
     </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="n">
         <v>44</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C45" s="9" t="s">
         <v>266</v>
@@ -3829,7 +3829,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>271</v>
@@ -3854,7 +3854,7 @@
         <v>275</v>
       </c>
       <c r="K46" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L46" s="9"/>
       <c r="M46" s="10"/>
@@ -3865,7 +3865,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C47" s="9" t="s">
         <v>276</v>
@@ -3890,7 +3890,7 @@
         <v>280</v>
       </c>
       <c r="K47" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L47" s="9"/>
       <c r="M47" s="10"/>
@@ -3901,7 +3901,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C48" s="9" t="s">
         <v>281</v>
@@ -3926,7 +3926,7 @@
         <v>285</v>
       </c>
       <c r="K48" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L48" s="9"/>
       <c r="M48" s="10"/>
@@ -3937,7 +3937,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>286</v>
@@ -3960,7 +3960,7 @@
         <v>289</v>
       </c>
       <c r="K49" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L49" s="9"/>
       <c r="M49" s="10"/>
@@ -3971,7 +3971,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>290</v>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H50" s="9"/>
       <c r="I50" s="9" t="s">
@@ -3994,7 +3994,7 @@
         <v>292</v>
       </c>
       <c r="K50" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L50" s="9"/>
       <c r="M50" s="10"/>
@@ -4005,7 +4005,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C51" s="9" t="s">
         <v>293</v>
@@ -4030,7 +4030,7 @@
         <v>295</v>
       </c>
       <c r="K51" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L51" s="9"/>
       <c r="M51" s="10"/>
@@ -4041,7 +4041,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C52" s="9" t="s">
         <v>296</v>
@@ -4064,7 +4064,7 @@
         <v>298</v>
       </c>
       <c r="K52" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L52" s="9"/>
       <c r="M52" s="10"/>
@@ -4075,7 +4075,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C53" s="9" t="s">
         <v>299</v>
@@ -4091,7 +4091,7 @@
         <v>64</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I53" s="9" t="s">
         <v>202</v>
@@ -4100,7 +4100,7 @@
         <v>302</v>
       </c>
       <c r="K53" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L53" s="9"/>
       <c r="M53" s="10"/>
@@ -4111,13 +4111,13 @@
         <v>53</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E54" s="9" t="s">
         <v>303</v>
@@ -4127,7 +4127,7 @@
         <v>64</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I54" s="9" t="s">
         <v>202</v>
@@ -4136,7 +4136,7 @@
         <v>304</v>
       </c>
       <c r="K54" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L54" s="9"/>
       <c r="M54" s="10"/>
@@ -4147,13 +4147,13 @@
         <v>54</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>305</v>
@@ -4163,7 +4163,7 @@
         <v>64</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I55" s="9" t="s">
         <v>202</v>
@@ -4172,7 +4172,7 @@
         <v>306</v>
       </c>
       <c r="K55" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L55" s="9"/>
       <c r="M55" s="10"/>
@@ -4183,7 +4183,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C56" s="9" t="s">
         <v>307</v>
@@ -4206,7 +4206,7 @@
         <v>310</v>
       </c>
       <c r="K56" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L56" s="9"/>
       <c r="M56" s="10"/>
@@ -4217,7 +4217,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C57" s="9" t="s">
         <v>311</v>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="F57" s="9"/>
       <c r="G57" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H57" s="9"/>
       <c r="I57" s="9" t="s">
@@ -4240,7 +4240,7 @@
         <v>315</v>
       </c>
       <c r="K57" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L57" s="9" t="s">
         <v>316</v>
@@ -4253,7 +4253,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C58" s="9" t="s">
         <v>317</v>
@@ -4276,7 +4276,7 @@
         <v>320</v>
       </c>
       <c r="K58" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L58" s="9"/>
       <c r="M58" s="10"/>
@@ -4287,7 +4287,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C59" s="9" t="s">
         <v>321</v>
@@ -4310,7 +4310,7 @@
         <v>324</v>
       </c>
       <c r="K59" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L59" s="9"/>
       <c r="M59" s="10"/>
@@ -4321,13 +4321,13 @@
         <v>59</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C60" s="9" t="s">
         <v>325</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E60" s="9" t="s">
         <v>326</v>
@@ -4337,7 +4337,7 @@
         <v>64</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I60" s="9" t="s">
         <v>202</v>
@@ -4346,7 +4346,7 @@
         <v>327</v>
       </c>
       <c r="K60" s="9" t="s">
-        <v>66</v>
+        <v>129</v>
       </c>
       <c r="L60" s="9"/>
       <c r="M60" s="10"/>
@@ -4357,13 +4357,13 @@
         <v>60</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C61" s="9" t="s">
         <v>328</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>329</v>
@@ -4373,7 +4373,7 @@
         <v>64</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I61" s="9" t="s">
         <v>7</v>
@@ -4382,7 +4382,7 @@
         <v>330</v>
       </c>
       <c r="K61" s="9" t="s">
-        <v>66</v>
+        <v>129</v>
       </c>
       <c r="L61" s="9"/>
       <c r="M61" s="10"/>
@@ -4393,13 +4393,13 @@
         <v>61</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C62" s="9" t="s">
         <v>331</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E62" s="9" t="s">
         <v>332</v>
@@ -4418,7 +4418,7 @@
         <v>333</v>
       </c>
       <c r="K62" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L62" s="9"/>
       <c r="M62" s="10"/>
@@ -4429,7 +4429,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C63" s="9" t="s">
         <v>334</v>
@@ -4452,7 +4452,7 @@
         <v>337</v>
       </c>
       <c r="K63" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L63" s="9"/>
       <c r="M63" s="10"/>
@@ -4463,7 +4463,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C64" s="9" t="s">
         <v>338</v>
@@ -4486,7 +4486,7 @@
         <v>341</v>
       </c>
       <c r="K64" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L64" s="9"/>
       <c r="M64" s="10"/>
@@ -4497,7 +4497,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C65" s="9" t="s">
         <v>342</v>
@@ -4520,7 +4520,7 @@
         <v>345</v>
       </c>
       <c r="K65" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L65" s="9"/>
       <c r="M65" s="10"/>
@@ -4531,7 +4531,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C66" s="9" t="s">
         <v>346</v>
@@ -4554,7 +4554,7 @@
         <v>348</v>
       </c>
       <c r="K66" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L66" s="9"/>
       <c r="M66" s="10"/>
@@ -4565,7 +4565,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C67" s="9" t="s">
         <v>233</v>
@@ -4590,7 +4590,7 @@
         <v>351</v>
       </c>
       <c r="K67" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L67" s="9"/>
       <c r="M67" s="10"/>
@@ -4601,7 +4601,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C68" s="9" t="s">
         <v>352</v>
@@ -4617,7 +4617,7 @@
         <v>64</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I68" s="9" t="s">
         <v>7</v>
@@ -4626,7 +4626,7 @@
         <v>355</v>
       </c>
       <c r="K68" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L68" s="9"/>
       <c r="M68" s="10"/>
@@ -4637,7 +4637,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C69" s="9" t="s">
         <v>356</v>
@@ -4653,7 +4653,7 @@
         <v>64</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I69" s="9" t="s">
         <v>202</v>
@@ -4662,7 +4662,7 @@
         <v>358</v>
       </c>
       <c r="K69" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L69" s="9"/>
       <c r="M69" s="10"/>
@@ -4673,7 +4673,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C70" s="9" t="s">
         <v>274</v>
@@ -4698,7 +4698,7 @@
         <v>361</v>
       </c>
       <c r="K70" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L70" s="9"/>
       <c r="M70" s="10"/>
@@ -4709,7 +4709,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C71" s="9" t="s">
         <v>279</v>
@@ -4734,7 +4734,7 @@
         <v>363</v>
       </c>
       <c r="K71" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L71" s="9"/>
       <c r="M71" s="10"/>
@@ -4745,7 +4745,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C72" s="9" t="s">
         <v>284</v>
@@ -4770,7 +4770,7 @@
         <v>365</v>
       </c>
       <c r="K72" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L72" s="9"/>
       <c r="M72" s="10"/>
@@ -4781,7 +4781,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C73" s="9" t="s">
         <v>366</v>
@@ -4804,7 +4804,7 @@
         <v>369</v>
       </c>
       <c r="K73" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L73" s="9"/>
       <c r="M73" s="10"/>
@@ -4815,13 +4815,13 @@
         <v>73</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C74" s="9" t="s">
         <v>370</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E74" s="9" t="s">
         <v>371</v>
@@ -4838,7 +4838,7 @@
         <v>372</v>
       </c>
       <c r="K74" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L74" s="9"/>
       <c r="M74" s="10"/>
@@ -4849,7 +4849,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C75" s="9" t="s">
         <v>373</v>
@@ -4874,7 +4874,7 @@
         <v>242</v>
       </c>
       <c r="K75" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L75" s="9"/>
       <c r="M75" s="10"/>
@@ -4885,7 +4885,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C76" s="9" t="s">
         <v>375</v>
@@ -4910,7 +4910,7 @@
         <v>376</v>
       </c>
       <c r="K76" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L76" s="9"/>
       <c r="M76" s="10"/>
@@ -4921,7 +4921,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C77" s="9" t="s">
         <v>188</v>
@@ -4946,7 +4946,7 @@
         <v>378</v>
       </c>
       <c r="K77" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L77" s="9"/>
       <c r="M77" s="10"/>
@@ -4957,7 +4957,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C78" s="9" t="s">
         <v>379</v>
@@ -4982,7 +4982,7 @@
         <v>383</v>
       </c>
       <c r="K78" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L78" s="9"/>
       <c r="M78" s="10"/>
@@ -4993,7 +4993,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C79" s="9" t="s">
         <v>384</v>
@@ -5018,7 +5018,7 @@
         <v>386</v>
       </c>
       <c r="K79" s="9" t="s">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="L79" s="9"/>
       <c r="M79" s="10"/>
@@ -5029,7 +5029,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C80" s="9" t="s">
         <v>382</v>
@@ -5054,7 +5054,7 @@
         <v>387</v>
       </c>
       <c r="K80" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L80" s="9"/>
       <c r="M80" s="10"/>
@@ -5065,7 +5065,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C81" s="9" t="s">
         <v>388</v>
@@ -5088,7 +5088,7 @@
         <v>391</v>
       </c>
       <c r="K81" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L81" s="9"/>
       <c r="M81" s="10"/>
@@ -5099,7 +5099,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C82" s="9" t="s">
         <v>392</v>
@@ -5122,7 +5122,7 @@
         <v>394</v>
       </c>
       <c r="K82" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L82" s="9"/>
       <c r="M82" s="10"/>
@@ -5133,7 +5133,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C83" s="9" t="s">
         <v>395</v>
@@ -5169,7 +5169,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C84" s="9" t="s">
         <v>403</v>
@@ -5205,7 +5205,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C85" s="9" t="s">
         <v>407</v>
@@ -5221,7 +5221,7 @@
         <v>64</v>
       </c>
       <c r="H85" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I85" s="9" t="s">
         <v>202</v>
@@ -5230,7 +5230,7 @@
         <v>302</v>
       </c>
       <c r="K85" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L85" s="9"/>
       <c r="M85" s="10"/>
@@ -5241,7 +5241,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C86" s="9" t="s">
         <v>410</v>
@@ -5277,7 +5277,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C87" s="9" t="s">
         <v>415</v>
@@ -5311,7 +5311,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C88" s="9" t="s">
         <v>419</v>
@@ -5327,7 +5327,7 @@
         <v>64</v>
       </c>
       <c r="H88" s="9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I88" s="9" t="s">
         <v>202</v>
@@ -5336,7 +5336,7 @@
         <v>203</v>
       </c>
       <c r="K88" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L88" s="9"/>
       <c r="M88" s="10"/>
@@ -5347,7 +5347,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C89" s="9" t="s">
         <v>422</v>
@@ -5372,7 +5372,7 @@
         <v>425</v>
       </c>
       <c r="K89" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L89" s="9"/>
       <c r="M89" s="10"/>
@@ -5383,13 +5383,13 @@
         <v>89</v>
       </c>
       <c r="B90" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C90" s="9" t="s">
         <v>426</v>
       </c>
       <c r="D90" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E90" s="9" t="s">
         <v>427</v>
@@ -5406,7 +5406,7 @@
         <v>428</v>
       </c>
       <c r="K90" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L90" s="9"/>
       <c r="M90" s="10"/>
@@ -5417,13 +5417,13 @@
         <v>90</v>
       </c>
       <c r="B91" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C91" s="9" t="s">
         <v>429</v>
       </c>
       <c r="D91" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>430</v>
@@ -5442,7 +5442,7 @@
         <v>431</v>
       </c>
       <c r="K91" s="9" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L91" s="9"/>
       <c r="M91" s="10"/>

</xml_diff>